<commit_message>
added images for almost thirty frogs, and increased functionality for pages
</commit_message>
<xml_diff>
--- a/specieslist.xlsx
+++ b/specieslist.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drags\OSA_PiLA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OsaAnurans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F04AD0-7744-4AEF-826C-85DE5DD661E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="20715" windowHeight="13155"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>scientific_name</t>
   </si>
@@ -186,41 +185,14 @@
     <t>Lithobates warszewitschii</t>
   </si>
   <si>
-    <t>Bolitoglossa colonnea</t>
-  </si>
-  <si>
-    <t>Bolitoglossa lignicolor</t>
-  </si>
-  <si>
-    <t>Bolitoglossa schizodactyla</t>
-  </si>
-  <si>
-    <t>Oedipina alleni</t>
-  </si>
-  <si>
-    <t>Oedipina pacificensis</t>
-  </si>
-  <si>
-    <t>Oedipina savagei</t>
-  </si>
-  <si>
-    <t>Oscaecilia osae</t>
-  </si>
-  <si>
-    <t>Dermophis glandulosus</t>
-  </si>
-  <si>
-    <t>Dermophis occidentalis</t>
-  </si>
-  <si>
-    <t>Gymnopis multiplicata</t>
+    <t>display</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,6 +211,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -276,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -284,6 +264,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,329 +544,469 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A63"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B27" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A54" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A55" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A56" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A57" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A58" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A59" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A60" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A61" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A62" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A63" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changed pngs to webps and added common names in english
</commit_message>
<xml_diff>
--- a/specieslist.xlsx
+++ b/specieslist.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>scientific_name</t>
   </si>
@@ -186,13 +186,172 @@
   </si>
   <si>
     <t>display</t>
+  </si>
+  <si>
+    <t>common_name</t>
+  </si>
+  <si>
+    <t>Talamanca rocket frog</t>
+  </si>
+  <si>
+    <t>Variable harlequin toad</t>
+  </si>
+  <si>
+    <t>Pacific forest toad</t>
+  </si>
+  <si>
+    <t>Evergreen toad</t>
+  </si>
+  <si>
+    <t>Dark green toad</t>
+  </si>
+  <si>
+    <t>Truando toad</t>
+  </si>
+  <si>
+    <t>Cane toad</t>
+  </si>
+  <si>
+    <t>Grainy cochran frog</t>
+  </si>
+  <si>
+    <t>Emerald glass frog</t>
+  </si>
+  <si>
+    <t>Plantation glass frog</t>
+  </si>
+  <si>
+    <t>Fleischmann’s glass frog</t>
+  </si>
+  <si>
+    <t>La Palma glass frog</t>
+  </si>
+  <si>
+    <t>White-spotted Cochran frog</t>
+  </si>
+  <si>
+    <t>Chiriqui glass frog</t>
+  </si>
+  <si>
+    <t>Isla Bonita robber frog</t>
+  </si>
+  <si>
+    <t>Fitzinger's robber frog</t>
+  </si>
+  <si>
+    <t>Veragua robber frog</t>
+  </si>
+  <si>
+    <t>Stejneger's robber frog</t>
+  </si>
+  <si>
+    <t>South Pacific streamside frog</t>
+  </si>
+  <si>
+    <t>Chiriqui robber frog</t>
+  </si>
+  <si>
+    <t>Leopard robber frog</t>
+  </si>
+  <si>
+    <t>Rio San Juan robber frog</t>
+  </si>
+  <si>
+    <t>Green and black poison dart frog</t>
+  </si>
+  <si>
+    <t>Granular poison dart frog</t>
+  </si>
+  <si>
+    <t>Golfo Dulce poison dart frog</t>
+  </si>
+  <si>
+    <t>Rainforest rocket frog</t>
+  </si>
+  <si>
+    <t>Common dink frog</t>
+  </si>
+  <si>
+    <t>Vocal dink frog</t>
+  </si>
+  <si>
+    <t>Rosenberg's treefrog</t>
+  </si>
+  <si>
+    <t>Hourglass treefrog</t>
+  </si>
+  <si>
+    <t>Small-headed treefrog</t>
+  </si>
+  <si>
+    <t>Boulenger’s snouted treefrog</t>
+  </si>
+  <si>
+    <t>Sipurio snouted treefrog</t>
+  </si>
+  <si>
+    <t>Common Mexican treefrog</t>
+  </si>
+  <si>
+    <t>New Granada cross-banded treefrog</t>
+  </si>
+  <si>
+    <t>Panama cross-banded treefrog</t>
+  </si>
+  <si>
+    <t>Veragua cross-banded treefrog</t>
+  </si>
+  <si>
+    <t>Milk frog</t>
+  </si>
+  <si>
+    <t>Spiny-headed treefrog</t>
+  </si>
+  <si>
+    <t>Túngara frog</t>
+  </si>
+  <si>
+    <t>Bolivian white-lipped frog</t>
+  </si>
+  <si>
+    <t>American white-lipped frog</t>
+  </si>
+  <si>
+    <t>San Miguel island frog</t>
+  </si>
+  <si>
+    <t>Sabinal frog</t>
+  </si>
+  <si>
+    <t>Brown Foam-nest frog</t>
+  </si>
+  <si>
+    <t>Central American Bullfrog, Smoky Jungle frog</t>
+  </si>
+  <si>
+    <t>Costa Rica nelson frog</t>
+  </si>
+  <si>
+    <t>Colombian plump frog</t>
+  </si>
+  <si>
+    <t>Blue-sided treefrog</t>
+  </si>
+  <si>
+    <t>Red-eyed treefrog</t>
+  </si>
+  <si>
+    <t>Orange-sided gliding leaf frog</t>
+  </si>
+  <si>
+    <t>Brilliant Forest frog</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,16 +379,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -252,11 +430,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -265,6 +473,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,464 +759,623 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B27" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C28" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C30" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C34" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C35" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="65.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C36" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C37" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C38" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C39" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C40" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C41" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C42" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C43" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C44" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C45" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C46" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C47" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C48" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C49" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C50" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C51" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C52" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C53" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
     </row>
   </sheetData>

</xml_diff>